<commit_message>
test/checkout-update checkout test cases
</commit_message>
<xml_diff>
--- a/TestCases_Docs/CHK_TCS.xlsx
+++ b/TestCases_Docs/CHK_TCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FOTOH_COMPU\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E2137E5-268D-43FE-B4FB-3E266F2A33C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4016CC12-938D-4401-8881-2C0C96DDB7D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="310">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>TC_CHK_001</t>
-  </si>
-  <si>
-    <t>Verify successful checkout with valid data</t>
   </si>
   <si>
     <t>Web / Chrome</t>
@@ -93,60 +90,19 @@
 User logged in</t>
   </si>
   <si>
-    <t>1. Select product from home page 
-2. Add product to cart
-3. Open cart 
-4. Click checkout
-5. Enter City 
-6. Enter Address 
-7. Click Confirm Order</t>
-  </si>
-  <si>
-    <t>City: Cairo, Address: Nasr City</t>
-  </si>
-  <si>
-    <t>Order is placed successfully and 
-user is redirected to home page</t>
-  </si>
-  <si>
-    <t>Order completed successfully</t>
-  </si>
-  <si>
     <t>in review</t>
   </si>
   <si>
     <t>N/A</t>
   </si>
   <si>
-    <t>End-to-End</t>
-  </si>
-  <si>
     <t>Hager Elwan</t>
   </si>
   <si>
     <t>TC_CHK_002</t>
   </si>
   <si>
-    <t>Verify checkout page displays all required elements</t>
-  </si>
-  <si>
-    <t>1. Open checkout page 
-2. Verify City field 
-3. Verify Address field 
-4. Verify Cash on Delivery text 
-5. Verify Confirm Order button</t>
-  </si>
-  <si>
-    <t>All required checkout elements are displayed correctly</t>
-  </si>
-  <si>
-    <t>Checkout page remains open</t>
-  </si>
-  <si>
     <t>TC_CHK_003</t>
-  </si>
-  <si>
-    <t>Verify City field is mandatory</t>
   </si>
   <si>
     <t xml:space="preserve">open URL
@@ -154,44 +110,10 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">
-1. Select product from home page 
-2. Add product to cart
-3. Open cart 
-4. Click checkout
-5. Leave City Empty  
-6. Enter Address 
-6. Click Confirm Order</t>
-  </si>
-  <si>
-    <t>City: Empty, Address: Dokki</t>
-  </si>
-  <si>
     <t>User stays on checkout page</t>
   </si>
   <si>
     <t>TC_CHK_005</t>
-  </si>
-  <si>
-    <t>Verify user cannot proceed to checkout with empty cart</t>
-  </si>
-  <si>
-    <t>open URL
-User logged in with empty cart</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1.Open cart 
-2. Click checkout</t>
-  </si>
-  <si>
-    <t>Empty cart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User cannot proceed to checkout 
-</t>
-  </si>
-  <si>
-    <t>User remains on cart page</t>
   </si>
   <si>
     <t>TC_CHK_006</t>
@@ -212,37 +134,16 @@
     <t>Guest user</t>
   </si>
   <si>
-    <t xml:space="preserve">User is redirected to login </t>
-  </si>
-  <si>
     <t>User lands on login page</t>
   </si>
   <si>
-    <t xml:space="preserve">Validation message appears and order is not placed
-</t>
-  </si>
-  <si>
     <t>TC_CHK_007</t>
   </si>
   <si>
     <t>Verify confirmation email is sent to the customer after placing order</t>
   </si>
   <si>
-    <t>1.Select product from home page 
-2. Add product to cart 
-3. Open cart 
-4. Click checkout 
-5. Enter City 
-6. Enter Address 
-7. Click Place Order 
-8. Check customer email</t>
-  </si>
-  <si>
     <t>A confirmation email is sent to the customer after successful order placement</t>
-  </si>
-  <si>
-    <t>Order is completed 
-and confirmation email is received</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -1348,42 +1249,197 @@
     <t>SIQ_Acc_09</t>
   </si>
   <si>
-    <t>SRS-FN-CHK-002</t>
-  </si>
-  <si>
-    <t>Verify Adress field is mandatory</t>
-  </si>
-  <si>
     <t>TC_CHK_004</t>
   </si>
   <si>
-    <t xml:space="preserve">
-1. Select product from home page 
+    <t>SRS-FN-Checkout-005</t>
+  </si>
+  <si>
+    <t>SRS-FN-Checkout-002</t>
+  </si>
+  <si>
+    <t>SRS-FN- Checkout-001</t>
+  </si>
+  <si>
+    <t>pop up message "Order is placed successfully"
+and 
+user is redirected to home page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pop up message appears
+"Please Enter the required data"
+ and order is not placed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-FN-Checkout-002
+</t>
+  </si>
+  <si>
+    <t>pop up message appears
+"Please Enter the required data"
+ and order is not placed</t>
+  </si>
+  <si>
+    <t>Order Submitted successfully and redirect customer to home page</t>
+  </si>
+  <si>
+    <t>Validate that all checkout page input fields are labeled</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
 2. Add product to cart
 3. Open cart 
 4. Click checkout
-5. Enter City   
-6. Leave Address empty
-6. Click Confirm Order</t>
-  </si>
-  <si>
-    <t>City: cairo, Address: Empty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-FN-CHK-003
-SRS-FN-CHK-004
+5.Observe all input fields on the checkout page
+6.Check that each input field has a clear
+ and visible label</t>
+  </si>
+  <si>
+    <t>All input fields on the checkout page are displayed with correct, clear, and visible labels.</t>
+  </si>
+  <si>
+    <t>Checkout page remains displayed with all input fields and labels visible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify successful checkout with valid data
+(city, Address, Mobile phone of reciever, name's reciever) </t>
+  </si>
+  <si>
+    <t>Verify Address field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t>Verify name of reciever field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t>Verify City field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify phone of reciever field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field empty
+6. Enter Address field empty
+7. Leave phone of reciever
+8.Enter name of reciever empty
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field empty
+6. Enter Address field empty
+7. Enter phone of reciever
+8.leave name of reciever empty
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field empty
+6. Leave Address field empty
+7. Enter phone of reciever
+8.Enter name of reciever
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Leave City field empty
+6. Enter Address 
+7. Enter phone of reciever
+8.Enter name of reciever
+9. Click confirm Order button
 </t>
   </si>
   <si>
-    <t xml:space="preserve">SRS-FN-CHK-006
-</t>
-  </si>
-  <si>
-    <t>SRS-FN-CHK-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS-FN-CHK-001
-</t>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City 
+6. Enter Address 
+7. Enter phone of reciever
+8.Enter name of reciever
+9. Click confirm Order button
+10.redirect to home page</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field empty
+6. Enter Address field empty
+7. Enter phone of reciever
+8.Enter name of reciever empty
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>The Confirm Order button is displayed on the checkout page and clickable when entered valid data</t>
+  </si>
+  <si>
+    <t>pop up message appears
+"Ple+I8+H8+H8:H10</t>
+  </si>
+  <si>
+    <t>Order Submitted successfully
+ and redirect customer
+ to home page</t>
+  </si>
+  <si>
+    <t>SRS-FN- Checkout-003</t>
+  </si>
+  <si>
+    <t>Verify that the "Confirm Order" button is displayed and clickable to confirm the order</t>
+  </si>
+  <si>
+    <t>TC_CHK_008</t>
+  </si>
+  <si>
+    <t>Verify Cash on Delivery (COD) payment method is clearly displayed as text  on checkout page</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5.Observe the payment method section on the is displayed as text checkout page</t>
+  </si>
+  <si>
+    <t>The system clearly displays Cash on Delivery (COD) as the payment method on the checkout page</t>
+  </si>
+  <si>
+    <t>Checkout page remains displayed with COD payment method visible.</t>
+  </si>
+  <si>
+    <t>SRS-FN-Checkout-004</t>
+  </si>
+  <si>
+    <t>TC_CHK_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is redirected to login page </t>
+  </si>
+  <si>
+    <t>TC_CHK_010</t>
+  </si>
+  <si>
+    <t>Order is submitted 
+and confirmation email is received</t>
+  </si>
+  <si>
+    <t>SRS-FN-Checkout-006</t>
   </si>
 </sst>
 </file>
@@ -1522,7 +1578,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1622,6 +1678,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1844,18 +1903,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA978"/>
+  <dimension ref="A1:AA981"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7265625" customWidth="1"/>
-    <col min="2" max="2" width="111.453125" customWidth="1"/>
+    <col min="2" max="2" width="123.6328125" customWidth="1"/>
     <col min="3" max="3" width="21.26953125" customWidth="1"/>
     <col min="4" max="4" width="18.26953125" customWidth="1"/>
     <col min="5" max="5" width="56.36328125" customWidth="1"/>
     <col min="6" max="6" width="41.453125" customWidth="1"/>
     <col min="7" max="7" width="32.6328125" customWidth="1"/>
     <col min="8" max="8" width="40.7265625" customWidth="1"/>
-    <col min="9" max="10" width="18.26953125" customWidth="1"/>
+    <col min="9" max="9" width="26.36328125" customWidth="1"/>
+    <col min="10" max="10" width="18.26953125" customWidth="1"/>
     <col min="11" max="11" width="16.6328125" customWidth="1"/>
     <col min="12" max="12" width="24" customWidth="1"/>
     <col min="13" max="27" width="18.26953125" customWidth="1"/>
@@ -1908,463 +1968,486 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="87.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" ht="125" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>20</v>
+      <c r="B2" s="22" t="s">
+        <v>283</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D2" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="F2" s="22" t="s">
+        <v>292</v>
+      </c>
+      <c r="G2" s="14"/>
+      <c r="H2" s="23" t="s">
+        <v>274</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>278</v>
+      </c>
+      <c r="J2" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="K2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="13" t="s">
+      <c r="L2" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="M2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="103" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="K2" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>299</v>
-      </c>
-      <c r="M2" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="62.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>32</v>
+      <c r="B3" s="22" t="s">
+        <v>279</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D3" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="F3" s="22" t="s">
+        <v>280</v>
+      </c>
+      <c r="G3" s="14"/>
+      <c r="H3" s="23" t="s">
+        <v>281</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="J3" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>28</v>
-      </c>
+      <c r="K3" s="14"/>
       <c r="L3" s="23" t="s">
-        <v>298</v>
-      </c>
-      <c r="M3" s="14"/>
-      <c r="N3" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" ht="100" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+      <c r="M3" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="N3" s="13"/>
+    </row>
+    <row r="4" spans="1:27" ht="125" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>37</v>
+        <v>286</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>56</v>
+        <v>291</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="23" t="s">
+        <v>275</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="M4" s="14"/>
+        <v>23</v>
+      </c>
+      <c r="L4" s="23" t="s">
+        <v>276</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>16</v>
+      </c>
       <c r="N4" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" ht="100" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>295</v>
+        <v>270</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>38</v>
+        <v>20</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>27</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>296</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>297</v>
-      </c>
+        <v>290</v>
+      </c>
+      <c r="G5" s="14"/>
       <c r="H5" s="23" t="s">
-        <v>56</v>
+        <v>277</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="M5" s="14"/>
+        <v>272</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>16</v>
+      </c>
       <c r="N5" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" ht="25" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" ht="133.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>43</v>
+        <v>285</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>44</v>
-      </c>
       <c r="F6" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>47</v>
+        <v>289</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="23" t="s">
+        <v>277</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="L6" s="23" t="s">
-        <v>301</v>
+        <v>22</v>
+      </c>
+      <c r="K6" s="14"/>
+      <c r="L6" s="13" t="s">
+        <v>272</v>
       </c>
       <c r="M6" s="14" t="s">
         <v>16</v>
       </c>
       <c r="N6" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>49</v>
-      </c>
       <c r="B7" s="14" t="s">
-        <v>50</v>
+        <v>287</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>51</v>
-      </c>
       <c r="F7" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>54</v>
+        <v>288</v>
+      </c>
+      <c r="G7" s="14"/>
+      <c r="H7" s="23" t="s">
+        <v>295</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="L7" s="23" t="s">
-        <v>299</v>
+        <v>22</v>
+      </c>
+      <c r="K7" s="14"/>
+      <c r="L7" s="13" t="s">
+        <v>272</v>
       </c>
       <c r="M7" s="14" t="s">
         <v>16</v>
       </c>
       <c r="N7" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" ht="100" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>58</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>298</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="22" t="s">
+        <v>293</v>
+      </c>
+      <c r="G8" s="14"/>
+      <c r="H8" s="23" t="s">
+        <v>294</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>296</v>
+      </c>
+      <c r="J8" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="K8" s="14"/>
+      <c r="L8" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="M8" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="N8" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:27" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>299</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="C9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>301</v>
+      </c>
+      <c r="G9" s="14"/>
+      <c r="H9" s="23" t="s">
+        <v>302</v>
+      </c>
+      <c r="I9" s="22" t="s">
+        <v>303</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="14"/>
+      <c r="L9" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="M9" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2"/>
-      <c r="AA8" s="2"/>
-    </row>
-    <row r="9" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="7"/>
-      <c r="S9" s="7"/>
-      <c r="T9" s="7"/>
-      <c r="U9" s="7"/>
-      <c r="V9" s="7"/>
-      <c r="W9" s="7"/>
-      <c r="X9" s="7"/>
-      <c r="Y9" s="7"/>
-      <c r="Z9" s="7"/>
-      <c r="AA9" s="7"/>
-    </row>
-    <row r="10" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="8"/>
-      <c r="AA10" s="8"/>
-    </row>
-    <row r="11" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11"/>
-      <c r="S11" s="11"/>
-      <c r="T11" s="11"/>
-      <c r="U11" s="11"/>
-      <c r="V11" s="11"/>
-      <c r="W11" s="11"/>
-      <c r="X11" s="11"/>
-      <c r="Y11" s="11"/>
-      <c r="Z11" s="11"/>
-      <c r="AA11" s="11"/>
+      <c r="N9" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="L10" s="23" t="s">
+        <v>271</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="N10" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2"/>
+      <c r="Z11" s="2"/>
+      <c r="AA11" s="2"/>
     </row>
     <row r="12" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="11"/>
-      <c r="W12" s="11"/>
-      <c r="X12" s="11"/>
-      <c r="Y12" s="11"/>
-      <c r="Z12" s="11"/>
-      <c r="AA12" s="11"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="7"/>
+      <c r="X12" s="7"/>
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="7"/>
+      <c r="AA12" s="7"/>
     </row>
     <row r="13" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
       <c r="C13" s="9"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="11"/>
-      <c r="W13" s="11"/>
-      <c r="X13" s="11"/>
-      <c r="Y13" s="11"/>
-      <c r="Z13" s="11"/>
-      <c r="AA13" s="11"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
+      <c r="AA13" s="8"/>
     </row>
     <row r="14" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
@@ -2454,268 +2537,291 @@
       <c r="AA16" s="11"/>
     </row>
     <row r="17" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C17" s="2"/>
-      <c r="H17" s="13"/>
-      <c r="J17" s="14"/>
-      <c r="L17" s="13"/>
-      <c r="N17" s="13"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="11"/>
+      <c r="T17" s="11"/>
+      <c r="U17" s="11"/>
+      <c r="V17" s="11"/>
+      <c r="W17" s="11"/>
+      <c r="X17" s="11"/>
+      <c r="Y17" s="11"/>
+      <c r="Z17" s="11"/>
+      <c r="AA17" s="11"/>
     </row>
     <row r="18" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C18" s="2"/>
-      <c r="H18" s="13"/>
-      <c r="J18" s="14"/>
-      <c r="L18" s="13"/>
-      <c r="N18" s="13"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="11"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="11"/>
+      <c r="S18" s="11"/>
+      <c r="T18" s="11"/>
+      <c r="U18" s="11"/>
+      <c r="V18" s="11"/>
+      <c r="W18" s="11"/>
+      <c r="X18" s="11"/>
+      <c r="Y18" s="11"/>
+      <c r="Z18" s="11"/>
+      <c r="AA18" s="11"/>
     </row>
     <row r="19" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C19" s="2"/>
-      <c r="H19" s="13"/>
-      <c r="J19" s="14"/>
-      <c r="L19" s="13"/>
-      <c r="N19" s="13"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="11"/>
+      <c r="Q19" s="11"/>
+      <c r="R19" s="11"/>
+      <c r="S19" s="11"/>
+      <c r="T19" s="11"/>
+      <c r="U19" s="11"/>
+      <c r="V19" s="11"/>
+      <c r="W19" s="11"/>
+      <c r="X19" s="11"/>
+      <c r="Y19" s="11"/>
+      <c r="Z19" s="11"/>
+      <c r="AA19" s="11"/>
     </row>
     <row r="20" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="16"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
-      <c r="S20" s="15"/>
-      <c r="T20" s="15"/>
-      <c r="U20" s="15"/>
-      <c r="V20" s="15"/>
-      <c r="W20" s="15"/>
-      <c r="X20" s="15"/>
-      <c r="Y20" s="15"/>
-      <c r="Z20" s="15"/>
-      <c r="AA20" s="15"/>
-    </row>
-    <row r="21" spans="1:27" ht="14" x14ac:dyDescent="0.25">
-      <c r="A21" s="17"/>
-      <c r="B21" s="17"/>
+      <c r="C20" s="2"/>
+      <c r="H20" s="13"/>
+      <c r="J20" s="14"/>
+      <c r="L20" s="13"/>
+      <c r="N20" s="13"/>
+    </row>
+    <row r="21" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C21" s="2"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="20"/>
-      <c r="P21" s="20"/>
-      <c r="Q21" s="20"/>
-      <c r="R21" s="20"/>
-      <c r="S21" s="20"/>
-      <c r="T21" s="20"/>
-      <c r="U21" s="20"/>
-      <c r="V21" s="20"/>
-      <c r="W21" s="20"/>
-      <c r="X21" s="20"/>
-      <c r="Y21" s="20"/>
-      <c r="Z21" s="20"/>
-      <c r="AA21" s="20"/>
+      <c r="H21" s="13"/>
+      <c r="J21" s="14"/>
+      <c r="L21" s="13"/>
+      <c r="N21" s="13"/>
     </row>
     <row r="22" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C22" s="2"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="23"/>
+      <c r="H22" s="13"/>
+      <c r="J22" s="14"/>
       <c r="L22" s="13"/>
       <c r="N22" s="13"/>
     </row>
     <row r="23" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C23" s="2"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="23"/>
-      <c r="L23" s="13"/>
-      <c r="N23" s="13"/>
-    </row>
-    <row r="24" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="15"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="15"/>
+      <c r="P23" s="15"/>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="15"/>
+      <c r="T23" s="15"/>
+      <c r="U23" s="15"/>
+      <c r="V23" s="15"/>
+      <c r="W23" s="15"/>
+      <c r="X23" s="15"/>
+      <c r="Y23" s="15"/>
+      <c r="Z23" s="15"/>
+      <c r="AA23" s="15"/>
+    </row>
+    <row r="24" spans="1:27" ht="14" x14ac:dyDescent="0.25">
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="2"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="H24" s="23"/>
-      <c r="L24" s="13"/>
-      <c r="N24" s="13"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="21"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="18"/>
+      <c r="O24" s="20"/>
+      <c r="P24" s="20"/>
+      <c r="Q24" s="20"/>
+      <c r="R24" s="20"/>
+      <c r="S24" s="20"/>
+      <c r="T24" s="20"/>
+      <c r="U24" s="20"/>
+      <c r="V24" s="20"/>
+      <c r="W24" s="20"/>
+      <c r="X24" s="20"/>
+      <c r="Y24" s="20"/>
+      <c r="Z24" s="20"/>
+      <c r="AA24" s="20"/>
     </row>
     <row r="25" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C25" s="2"/>
       <c r="E25" s="22"/>
       <c r="F25" s="22"/>
-      <c r="H25" s="2"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="23"/>
       <c r="L25" s="13"/>
       <c r="N25" s="13"/>
     </row>
     <row r="26" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="16"/>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="15"/>
-      <c r="R26" s="15"/>
-      <c r="S26" s="15"/>
-      <c r="T26" s="15"/>
-      <c r="U26" s="15"/>
-      <c r="V26" s="15"/>
-      <c r="W26" s="15"/>
-      <c r="X26" s="15"/>
-      <c r="Y26" s="15"/>
-      <c r="Z26" s="15"/>
-      <c r="AA26" s="15"/>
-    </row>
-    <row r="27" spans="1:27" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13"/>
+      <c r="C26" s="2"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="23"/>
+      <c r="L26" s="13"/>
+      <c r="N26" s="13"/>
+    </row>
+    <row r="27" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C27" s="2"/>
-      <c r="H27" s="13"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="H27" s="23"/>
       <c r="L27" s="13"/>
       <c r="N27" s="13"/>
     </row>
-    <row r="28" spans="1:27" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C28" s="2"/>
-      <c r="H28" s="13"/>
-      <c r="J28" s="14"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="H28" s="2"/>
       <c r="L28" s="13"/>
       <c r="N28" s="13"/>
     </row>
-    <row r="29" spans="1:27" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="2"/>
-      <c r="H29" s="13"/>
-      <c r="J29" s="14"/>
-      <c r="L29" s="13"/>
-      <c r="N29" s="13"/>
-    </row>
-    <row r="30" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15"/>
+      <c r="T29" s="15"/>
+      <c r="U29" s="15"/>
+      <c r="V29" s="15"/>
+      <c r="W29" s="15"/>
+      <c r="X29" s="15"/>
+      <c r="Y29" s="15"/>
+      <c r="Z29" s="15"/>
+      <c r="AA29" s="15"/>
+    </row>
+    <row r="30" spans="1:27" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13"/>
       <c r="C30" s="2"/>
       <c r="H30" s="13"/>
-      <c r="J30" s="14"/>
       <c r="L30" s="13"/>
       <c r="N30" s="13"/>
     </row>
-    <row r="31" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="2"/>
       <c r="H31" s="13"/>
       <c r="J31" s="14"/>
       <c r="L31" s="13"/>
       <c r="N31" s="13"/>
     </row>
-    <row r="32" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="2"/>
       <c r="H32" s="13"/>
       <c r="J32" s="14"/>
       <c r="L32" s="13"/>
       <c r="N32" s="13"/>
     </row>
-    <row r="33" spans="1:27" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C33" s="2"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="23"/>
+      <c r="H33" s="13"/>
       <c r="J33" s="14"/>
       <c r="L33" s="13"/>
       <c r="N33" s="13"/>
     </row>
-    <row r="34" spans="1:27" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="27"/>
+    <row r="34" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C34" s="2"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="28"/>
-      <c r="I34" s="27"/>
+      <c r="H34" s="13"/>
       <c r="J34" s="14"/>
-      <c r="K34" s="27"/>
-      <c r="L34" s="29"/>
-      <c r="M34" s="27"/>
-      <c r="N34" s="28"/>
-      <c r="O34" s="27"/>
-      <c r="P34" s="27"/>
-      <c r="Q34" s="27"/>
-      <c r="R34" s="27"/>
-      <c r="S34" s="27"/>
-      <c r="T34" s="27"/>
-      <c r="U34" s="27"/>
-      <c r="V34" s="27"/>
-      <c r="W34" s="27"/>
-      <c r="X34" s="27"/>
-      <c r="Y34" s="27"/>
-      <c r="Z34" s="27"/>
-      <c r="AA34" s="27"/>
-    </row>
-    <row r="35" spans="1:27" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="27"/>
+      <c r="L34" s="13"/>
+      <c r="N34" s="13"/>
+    </row>
+    <row r="35" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C35" s="2"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="27"/>
+      <c r="H35" s="13"/>
       <c r="J35" s="14"/>
-      <c r="K35" s="27"/>
-      <c r="L35" s="29"/>
-      <c r="M35" s="27"/>
-      <c r="N35" s="28"/>
-      <c r="O35" s="27"/>
-      <c r="P35" s="27"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="27"/>
-      <c r="S35" s="27"/>
-      <c r="T35" s="27"/>
-      <c r="U35" s="27"/>
-      <c r="V35" s="27"/>
-      <c r="W35" s="27"/>
-      <c r="X35" s="27"/>
-      <c r="Y35" s="27"/>
-      <c r="Z35" s="27"/>
-      <c r="AA35" s="27"/>
-    </row>
-    <row r="36" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="L35" s="13"/>
+      <c r="N35" s="13"/>
+    </row>
+    <row r="36" spans="1:27" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C36" s="2"/>
-      <c r="E36" s="14"/>
-      <c r="H36" s="13"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="23"/>
       <c r="J36" s="14"/>
-      <c r="L36" s="26"/>
+      <c r="L36" s="13"/>
       <c r="N36" s="13"/>
     </row>
-    <row r="37" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:27" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="27"/>
-      <c r="B37" s="27"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="30"/>
+      <c r="E37" s="27"/>
       <c r="F37" s="27"/>
       <c r="G37" s="27"/>
-      <c r="H37" s="31"/>
+      <c r="H37" s="28"/>
       <c r="I37" s="27"/>
       <c r="J37" s="14"/>
       <c r="K37" s="27"/>
@@ -2736,17 +2842,15 @@
       <c r="Z37" s="27"/>
       <c r="AA37" s="27"/>
     </row>
-    <row r="38" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:27" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="27"/>
-      <c r="B38" s="27"/>
       <c r="C38" s="2"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="30"/>
+      <c r="E38" s="27"/>
       <c r="F38" s="27"/>
       <c r="G38" s="27"/>
-      <c r="H38" s="31"/>
+      <c r="H38" s="28"/>
       <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
+      <c r="J38" s="14"/>
       <c r="K38" s="27"/>
       <c r="L38" s="29"/>
       <c r="M38" s="27"/>
@@ -2767,19 +2871,69 @@
     </row>
     <row r="39" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C39" s="2"/>
+      <c r="E39" s="14"/>
       <c r="H39" s="13"/>
       <c r="J39" s="14"/>
-      <c r="L39" s="13"/>
+      <c r="L39" s="26"/>
       <c r="N39" s="13"/>
     </row>
+    <row r="40" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="27"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="30"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="29"/>
+      <c r="M40" s="27"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="27"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
+      <c r="V40" s="27"/>
+      <c r="W40" s="27"/>
+      <c r="X40" s="27"/>
+      <c r="Y40" s="27"/>
+      <c r="Z40" s="27"/>
+      <c r="AA40" s="27"/>
+    </row>
     <row r="41" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C41" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H41" s="13"/>
-      <c r="J41" s="14"/>
-      <c r="L41" s="13"/>
-      <c r="N41" s="13"/>
+      <c r="A41" s="27"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="30"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="27"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="27"/>
+      <c r="L41" s="29"/>
+      <c r="M41" s="27"/>
+      <c r="N41" s="28"/>
+      <c r="O41" s="27"/>
+      <c r="P41" s="27"/>
+      <c r="Q41" s="27"/>
+      <c r="R41" s="27"/>
+      <c r="S41" s="27"/>
+      <c r="T41" s="27"/>
+      <c r="U41" s="27"/>
+      <c r="V41" s="27"/>
+      <c r="W41" s="27"/>
+      <c r="X41" s="27"/>
+      <c r="Y41" s="27"/>
+      <c r="Z41" s="27"/>
+      <c r="AA41" s="27"/>
     </row>
     <row r="42" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C42" s="2"/>
@@ -2788,15 +2942,10 @@
       <c r="L42" s="13"/>
       <c r="N42" s="13"/>
     </row>
-    <row r="43" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C43" s="2"/>
-      <c r="H43" s="13"/>
-      <c r="J43" s="14"/>
-      <c r="L43" s="13"/>
-      <c r="N43" s="13"/>
-    </row>
     <row r="44" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C44" s="2"/>
+      <c r="C44" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="H44" s="13"/>
       <c r="J44" s="14"/>
       <c r="L44" s="13"/>
@@ -2805,41 +2954,21 @@
     <row r="45" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C45" s="2"/>
       <c r="H45" s="13"/>
+      <c r="J45" s="14"/>
       <c r="L45" s="13"/>
       <c r="N45" s="13"/>
     </row>
     <row r="46" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A46" s="8"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="10"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
-      <c r="K46" s="8"/>
-      <c r="L46" s="10"/>
-      <c r="M46" s="8"/>
-      <c r="N46" s="10"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="8"/>
-      <c r="Q46" s="8"/>
-      <c r="R46" s="8"/>
-      <c r="S46" s="8"/>
-      <c r="T46" s="8"/>
-      <c r="U46" s="8"/>
-      <c r="V46" s="8"/>
-      <c r="W46" s="8"/>
-      <c r="X46" s="8"/>
-      <c r="Y46" s="8"/>
-      <c r="Z46" s="8"/>
-      <c r="AA46" s="8"/>
+      <c r="C46" s="2"/>
+      <c r="H46" s="13"/>
+      <c r="J46" s="14"/>
+      <c r="L46" s="13"/>
+      <c r="N46" s="13"/>
     </row>
     <row r="47" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C47" s="2"/>
       <c r="H47" s="13"/>
+      <c r="J47" s="14"/>
       <c r="L47" s="13"/>
       <c r="N47" s="13"/>
     </row>
@@ -2849,97 +2978,120 @@
       <c r="L48" s="13"/>
       <c r="N48" s="13"/>
     </row>
-    <row r="49" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C49" s="2"/>
-      <c r="H49" s="13"/>
-      <c r="L49" s="13"/>
-      <c r="N49" s="13"/>
-    </row>
-    <row r="50" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="8"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
+      <c r="L49" s="10"/>
+      <c r="M49" s="8"/>
+      <c r="N49" s="10"/>
+      <c r="O49" s="8"/>
+      <c r="P49" s="8"/>
+      <c r="Q49" s="8"/>
+      <c r="R49" s="8"/>
+      <c r="S49" s="8"/>
+      <c r="T49" s="8"/>
+      <c r="U49" s="8"/>
+      <c r="V49" s="8"/>
+      <c r="W49" s="8"/>
+      <c r="X49" s="8"/>
+      <c r="Y49" s="8"/>
+      <c r="Z49" s="8"/>
+      <c r="AA49" s="8"/>
+    </row>
+    <row r="50" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C50" s="2"/>
       <c r="H50" s="13"/>
       <c r="L50" s="13"/>
       <c r="N50" s="13"/>
     </row>
-    <row r="51" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C51" s="2"/>
       <c r="H51" s="13"/>
       <c r="L51" s="13"/>
       <c r="N51" s="13"/>
     </row>
-    <row r="52" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C52" s="2"/>
       <c r="H52" s="13"/>
       <c r="L52" s="13"/>
       <c r="N52" s="13"/>
     </row>
-    <row r="53" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C53" s="2"/>
       <c r="H53" s="13"/>
       <c r="L53" s="13"/>
       <c r="N53" s="13"/>
     </row>
-    <row r="54" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C54" s="2"/>
       <c r="H54" s="13"/>
       <c r="L54" s="13"/>
       <c r="N54" s="13"/>
     </row>
-    <row r="55" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C55" s="2"/>
       <c r="H55" s="13"/>
       <c r="L55" s="13"/>
       <c r="N55" s="13"/>
     </row>
-    <row r="56" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C56" s="2"/>
       <c r="H56" s="13"/>
       <c r="L56" s="13"/>
       <c r="N56" s="13"/>
     </row>
-    <row r="57" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C57" s="2"/>
       <c r="H57" s="13"/>
       <c r="L57" s="13"/>
       <c r="N57" s="13"/>
     </row>
-    <row r="58" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C58" s="2"/>
       <c r="H58" s="13"/>
       <c r="L58" s="13"/>
       <c r="N58" s="13"/>
     </row>
-    <row r="59" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C59" s="2"/>
       <c r="H59" s="13"/>
       <c r="L59" s="13"/>
       <c r="N59" s="13"/>
     </row>
-    <row r="60" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C60" s="2"/>
       <c r="H60" s="13"/>
       <c r="L60" s="13"/>
       <c r="N60" s="13"/>
     </row>
-    <row r="61" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C61" s="2"/>
       <c r="H61" s="13"/>
       <c r="L61" s="13"/>
       <c r="N61" s="13"/>
     </row>
-    <row r="62" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C62" s="2"/>
       <c r="H62" s="13"/>
       <c r="L62" s="13"/>
       <c r="N62" s="13"/>
     </row>
-    <row r="63" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C63" s="2"/>
       <c r="H63" s="13"/>
       <c r="L63" s="13"/>
       <c r="N63" s="13"/>
     </row>
-    <row r="64" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:27" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C64" s="2"/>
       <c r="H64" s="13"/>
       <c r="L64" s="13"/>
@@ -3144,16 +3296,19 @@
       <c r="N97" s="13"/>
     </row>
     <row r="98" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C98" s="2"/>
       <c r="H98" s="13"/>
       <c r="L98" s="13"/>
       <c r="N98" s="13"/>
     </row>
     <row r="99" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C99" s="2"/>
       <c r="H99" s="13"/>
       <c r="L99" s="13"/>
       <c r="N99" s="13"/>
     </row>
     <row r="100" spans="3:14" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="C100" s="2"/>
       <c r="H100" s="13"/>
       <c r="L100" s="13"/>
       <c r="N100" s="13"/>
@@ -7548,12 +7703,27 @@
       <c r="L978" s="13"/>
       <c r="N978" s="13"/>
     </row>
+    <row r="979" spans="8:14" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="H979" s="13"/>
+      <c r="L979" s="13"/>
+      <c r="N979" s="13"/>
+    </row>
+    <row r="980" spans="8:14" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="H980" s="13"/>
+      <c r="L980" s="13"/>
+      <c r="N980" s="13"/>
+    </row>
+    <row r="981" spans="8:14" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="H981" s="13"/>
+      <c r="L981" s="13"/>
+      <c r="N981" s="13"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C28:C39 C41:C44 C67:C97 C2:C19" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C31:C42 C44:C47 C70:C100 C2:C22" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"valid,invalid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J28:J39 J41:J44 J2:J19" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J31:J42 J44:J47 J2:J22" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"in progress,in review,approved,cancelled"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7594,7 +7764,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -7609,7 +7779,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="32" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -7633,54 +7803,54 @@
         <v>14</v>
       </c>
       <c r="Q1" s="32" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="99" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E2" s="33" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
@@ -7697,49 +7867,49 @@
     </row>
     <row r="3" spans="1:29" ht="50" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
@@ -7756,49 +7926,49 @@
     </row>
     <row r="4" spans="1:29" ht="100" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
@@ -7815,49 +7985,49 @@
     </row>
     <row r="5" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
@@ -7874,49 +8044,49 @@
     </row>
     <row r="6" spans="1:29" ht="100" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E6" s="34" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L6" s="4"/>
       <c r="M6" s="4" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
@@ -7933,49 +8103,49 @@
     </row>
     <row r="7" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="P7" s="2"/>
       <c r="Q7" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
@@ -7992,49 +8162,49 @@
     </row>
     <row r="8" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
@@ -8051,49 +8221,49 @@
     </row>
     <row r="9" spans="1:29" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L9" s="7"/>
       <c r="M9" s="4" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="P9" s="7"/>
       <c r="Q9" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
@@ -8110,47 +8280,47 @@
     </row>
     <row r="10" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
       <c r="K10" s="8" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L10" s="8"/>
       <c r="M10" s="10" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="P10" s="8"/>
       <c r="Q10" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R10" s="8"/>
       <c r="S10" s="8"/>
@@ -8167,47 +8337,47 @@
     </row>
     <row r="11" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="I11" s="11"/>
       <c r="J11" s="11"/>
       <c r="K11" s="11" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L11" s="11"/>
       <c r="M11" s="12" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="N11" s="11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O11" s="12" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="P11" s="11"/>
       <c r="Q11" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R11" s="11"/>
       <c r="S11" s="11"/>
@@ -8224,47 +8394,47 @@
     </row>
     <row r="12" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>130</v>
+        <v>107</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>18</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="I12" s="11"/>
       <c r="J12" s="11"/>
       <c r="K12" s="11" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L12" s="11"/>
       <c r="M12" s="12" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="N12" s="11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O12" s="12" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="P12" s="11"/>
       <c r="Q12" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R12" s="11"/>
       <c r="S12" s="11"/>
@@ -8281,47 +8451,47 @@
     </row>
     <row r="13" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>134</v>
+        <v>111</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I13" s="11"/>
       <c r="J13" s="11"/>
       <c r="K13" s="11" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L13" s="11"/>
       <c r="M13" s="12" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="N13" s="11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O13" s="12" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="P13" s="11"/>
       <c r="Q13" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R13" s="11"/>
       <c r="S13" s="11"/>
@@ -8338,47 +8508,47 @@
     </row>
     <row r="14" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I14" s="11"/>
       <c r="J14" s="11"/>
       <c r="K14" s="11" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L14" s="11"/>
       <c r="M14" s="12" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O14" s="12" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="P14" s="11"/>
       <c r="Q14" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R14" s="11"/>
       <c r="S14" s="11"/>
@@ -8395,47 +8565,47 @@
     </row>
     <row r="15" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I15" s="11"/>
       <c r="J15" s="11"/>
       <c r="K15" s="11" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L15" s="11"/>
       <c r="M15" s="12" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O15" s="12" t="s">
-        <v>142</v>
+        <v>119</v>
       </c>
       <c r="P15" s="11"/>
       <c r="Q15" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R15" s="11"/>
       <c r="S15" s="11"/>
@@ -8452,47 +8622,47 @@
     </row>
     <row r="16" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>144</v>
+        <v>121</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I16" s="11"/>
       <c r="J16" s="11"/>
       <c r="K16" s="11" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L16" s="11"/>
       <c r="M16" s="12" t="s">
-        <v>146</v>
+        <v>123</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O16" s="12" t="s">
-        <v>142</v>
+        <v>119</v>
       </c>
       <c r="P16" s="11"/>
       <c r="Q16" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R16" s="11"/>
       <c r="S16" s="11"/>
@@ -8509,192 +8679,192 @@
     </row>
     <row r="17" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>148</v>
+        <v>125</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="K17" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L17" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="M17" s="13" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="N17" s="14" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="O17" s="13" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>160</v>
+        <v>137</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="K18" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L18" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="N18" s="14" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="O18" s="13" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="K19" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L19" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="M19" s="13" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="N19" s="14" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="O19" s="13" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>168</v>
+        <v>145</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>169</v>
+        <v>146</v>
       </c>
       <c r="I20" s="15"/>
       <c r="J20" s="15" t="s">
-        <v>170</v>
+        <v>147</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>171</v>
+        <v>148</v>
       </c>
       <c r="N20" s="15" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O20" s="13" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="P20" s="15"/>
       <c r="Q20" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R20" s="15"/>
       <c r="S20" s="15"/>
@@ -8711,51 +8881,51 @@
     </row>
     <row r="21" spans="1:29" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>172</v>
+        <v>149</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>174</v>
+        <v>151</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>175</v>
+        <v>152</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>177</v>
+        <v>154</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="J21" s="20"/>
       <c r="K21" s="20" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L21" s="20"/>
       <c r="M21" s="21" t="s">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="N21" s="17" t="s">
         <v>16</v>
       </c>
       <c r="O21" s="18" t="s">
-        <v>180</v>
+        <v>157</v>
       </c>
       <c r="P21" s="35" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R21" s="20"/>
       <c r="S21" s="20"/>
@@ -8772,237 +8942,237 @@
     </row>
     <row r="22" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>183</v>
+        <v>160</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="K22" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M22" s="13" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="N22" s="14" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="P22" s="35" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>190</v>
+        <v>167</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>191</v>
+        <v>168</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="F23" s="24" t="s">
-        <v>192</v>
+        <v>169</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>193</v>
+        <v>170</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="K23" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="N23" s="14" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O23" s="13" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="P23" s="35" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:29" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>194</v>
+        <v>171</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>196</v>
+        <v>173</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>197</v>
+        <v>174</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>198</v>
+        <v>175</v>
       </c>
       <c r="H24" s="23" t="s">
-        <v>199</v>
+        <v>176</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="K24" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="N24" s="14" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O24" s="13"/>
       <c r="P24" s="35" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="Q24" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>202</v>
+        <v>179</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>203</v>
+        <v>180</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>204</v>
+        <v>181</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="I25" s="22" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="K25" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M25" s="13" t="s">
-        <v>206</v>
+        <v>183</v>
       </c>
       <c r="N25" s="14" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O25" s="13" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="P25" s="35" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>207</v>
+        <v>184</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>208</v>
+        <v>185</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E26" s="25" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="F26" s="25" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>210</v>
+        <v>187</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="I26" s="22" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="J26" s="15"/>
       <c r="K26" s="15" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="16" t="s">
-        <v>206</v>
+        <v>183</v>
       </c>
       <c r="N26" s="15" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O26" s="16" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="P26" s="35" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R26" s="15"/>
       <c r="S26" s="15"/>
@@ -9019,326 +9189,326 @@
     </row>
     <row r="27" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>211</v>
+        <v>188</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>212</v>
+        <v>189</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>213</v>
+        <v>190</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>214</v>
+        <v>191</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>215</v>
+        <v>192</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>216</v>
+        <v>193</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>217</v>
+        <v>194</v>
       </c>
       <c r="K27" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M27" s="13" t="s">
-        <v>218</v>
+        <v>195</v>
       </c>
       <c r="N27" s="14" t="s">
-        <v>219</v>
+        <v>196</v>
       </c>
       <c r="O27" s="13" t="s">
-        <v>220</v>
+        <v>197</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:29" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>221</v>
+        <v>198</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>213</v>
+        <v>190</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>225</v>
+        <v>202</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>226</v>
+        <v>203</v>
       </c>
       <c r="K28" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M28" s="13" t="s">
-        <v>218</v>
+        <v>195</v>
       </c>
       <c r="N28" s="14" t="s">
-        <v>219</v>
+        <v>196</v>
       </c>
       <c r="O28" s="13" t="s">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:29" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>228</v>
+        <v>205</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>213</v>
+        <v>190</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>230</v>
+        <v>207</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>231</v>
+        <v>208</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>232</v>
+        <v>209</v>
       </c>
       <c r="K29" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M29" s="13" t="s">
-        <v>233</v>
+        <v>210</v>
       </c>
       <c r="N29" s="14" t="s">
-        <v>219</v>
+        <v>196</v>
       </c>
       <c r="O29" s="13" t="s">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="Q29" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:29" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>234</v>
+        <v>211</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>235</v>
+        <v>212</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>236</v>
+        <v>213</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>237</v>
+        <v>214</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>238</v>
+        <v>215</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>239</v>
+        <v>216</v>
       </c>
       <c r="H30" s="23" t="s">
-        <v>240</v>
+        <v>217</v>
       </c>
       <c r="K30" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M30" s="13" t="s">
-        <v>241</v>
+        <v>218</v>
       </c>
       <c r="O30" s="13" t="s">
-        <v>242</v>
+        <v>219</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:29" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>243</v>
+        <v>220</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>244</v>
+        <v>221</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>236</v>
+        <v>213</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>245</v>
+        <v>222</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H31" s="23" t="s">
-        <v>246</v>
+        <v>223</v>
       </c>
       <c r="K31" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M31" s="13" t="s">
-        <v>241</v>
+        <v>218</v>
       </c>
       <c r="O31" s="13" t="s">
-        <v>242</v>
+        <v>219</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:29" ht="50" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>247</v>
+        <v>224</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>248</v>
+        <v>225</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>249</v>
+        <v>226</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>250</v>
+        <v>227</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>251</v>
+        <v>228</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>252</v>
+        <v>229</v>
       </c>
       <c r="H32" s="23" t="s">
-        <v>253</v>
+        <v>230</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>253</v>
+        <v>230</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="K32" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M32" s="13" t="s">
-        <v>241</v>
+        <v>218</v>
       </c>
       <c r="O32" s="13" t="s">
-        <v>254</v>
+        <v>231</v>
       </c>
       <c r="Q32" s="2" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33" spans="1:29" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>255</v>
+        <v>232</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>256</v>
+        <v>233</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>257</v>
+        <v>234</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>258</v>
+        <v>235</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>259</v>
+        <v>236</v>
       </c>
       <c r="G33" s="26" t="s">
-        <v>260</v>
+        <v>237</v>
       </c>
       <c r="H33" s="23" t="s">
-        <v>261</v>
+        <v>238</v>
       </c>
       <c r="J33" s="14" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="K33" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M33" s="13" t="s">
-        <v>263</v>
+        <v>240</v>
       </c>
       <c r="N33" s="14" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O33" s="13" t="s">
-        <v>264</v>
+        <v>241</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:29" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
-        <v>265</v>
+        <v>242</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>266</v>
+        <v>243</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>267</v>
+        <v>244</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>268</v>
+        <v>245</v>
       </c>
       <c r="G34" s="27" t="s">
-        <v>269</v>
+        <v>246</v>
       </c>
       <c r="H34" s="28" t="s">
-        <v>270</v>
+        <v>247</v>
       </c>
       <c r="I34" s="27"/>
       <c r="J34" s="27" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="K34" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L34" s="27"/>
       <c r="M34" s="29" t="s">
-        <v>271</v>
+        <v>248</v>
       </c>
       <c r="N34" s="27" t="s">
         <v>16</v>
@@ -9348,7 +9518,7 @@
       </c>
       <c r="P34" s="27"/>
       <c r="Q34" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R34" s="27"/>
       <c r="S34" s="27"/>
@@ -9365,39 +9535,39 @@
     </row>
     <row r="35" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="27" t="s">
-        <v>272</v>
+        <v>249</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>273</v>
+        <v>250</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E35" s="27" t="s">
-        <v>267</v>
+        <v>244</v>
       </c>
       <c r="F35" s="27" t="s">
-        <v>268</v>
+        <v>245</v>
       </c>
       <c r="G35" s="27" t="s">
-        <v>274</v>
+        <v>251</v>
       </c>
       <c r="H35" s="28" t="s">
-        <v>270</v>
+        <v>247</v>
       </c>
       <c r="I35" s="27"/>
       <c r="J35" s="27" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="K35" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L35" s="27"/>
       <c r="M35" s="29" t="s">
-        <v>271</v>
+        <v>248</v>
       </c>
       <c r="N35" s="27" t="s">
         <v>16</v>
@@ -9407,7 +9577,7 @@
       </c>
       <c r="P35" s="27"/>
       <c r="Q35" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R35" s="27"/>
       <c r="S35" s="27"/>
@@ -9424,37 +9594,37 @@
     </row>
     <row r="36" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>275</v>
+        <v>252</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>276</v>
+        <v>253</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E36" s="36" t="s">
-        <v>277</v>
+        <v>254</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>278</v>
+        <v>255</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>279</v>
+        <v>256</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>280</v>
+        <v>257</v>
       </c>
       <c r="J36" s="14" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="K36" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="M36" s="26" t="s">
-        <v>281</v>
+        <v>258</v>
       </c>
       <c r="N36" s="14" t="s">
         <v>16</v>
@@ -9463,54 +9633,54 @@
         <v>17</v>
       </c>
       <c r="Q36" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:29" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A37" s="27" t="s">
-        <v>282</v>
+        <v>259</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>283</v>
+        <v>260</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D37" s="27" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E37" s="30" t="s">
-        <v>267</v>
+        <v>244</v>
       </c>
       <c r="F37" s="27" t="s">
-        <v>284</v>
+        <v>261</v>
       </c>
       <c r="G37" s="27" t="s">
-        <v>285</v>
+        <v>262</v>
       </c>
       <c r="H37" s="31" t="s">
-        <v>286</v>
+        <v>263</v>
       </c>
       <c r="I37" s="27"/>
       <c r="J37" s="27" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="K37" s="14" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L37" s="27"/>
       <c r="M37" s="29" t="s">
-        <v>287</v>
+        <v>264</v>
       </c>
       <c r="N37" s="27" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O37" s="28" t="s">
-        <v>264</v>
+        <v>241</v>
       </c>
       <c r="P37" s="27"/>
       <c r="Q37" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R37" s="27"/>
       <c r="S37" s="27"/>
@@ -9527,49 +9697,49 @@
     </row>
     <row r="38" spans="1:29" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>289</v>
+        <v>266</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D38" s="27" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E38" s="30" t="s">
-        <v>258</v>
+        <v>235</v>
       </c>
       <c r="F38" s="27" t="s">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="G38" s="27" t="s">
-        <v>291</v>
+        <v>268</v>
       </c>
       <c r="H38" s="31" t="s">
-        <v>261</v>
+        <v>238</v>
       </c>
       <c r="I38" s="27"/>
       <c r="J38" s="27" t="s">
-        <v>262</v>
+        <v>239</v>
       </c>
       <c r="K38" s="27" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="L38" s="27"/>
       <c r="M38" s="29" t="s">
-        <v>292</v>
+        <v>269</v>
       </c>
       <c r="N38" s="27" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="O38" s="28" t="s">
-        <v>264</v>
+        <v>241</v>
       </c>
       <c r="P38" s="27"/>
       <c r="Q38" s="2" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="R38" s="27"/>
       <c r="S38" s="27"/>

</xml_diff>

<commit_message>
test/Updated Checkout Test Cases and Execution
</commit_message>
<xml_diff>
--- a/TestCases_Docs/CHK_TCS.xlsx
+++ b/TestCases_Docs/CHK_TCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CA0C588-050C-49B6-9B23-D0ED3BEEC6BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9236D6-EA61-4346-B3F3-1682EE664869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CHK_TCS" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="323">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1292,58 +1292,7 @@
     <t>Verify Address field is mandatory when left empty with other valid data</t>
   </si>
   <si>
-    <t>Verify name of reciever field is mandatory when left empty with other valid data</t>
-  </si>
-  <si>
     <t>Verify City field is mandatory when left empty with other valid data</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Verify phone of reciever field is mandatory when left empty with other valid data</t>
-  </si>
-  <si>
-    <t>1. Select product from home page 
-2. Add product to cart
-3. Open cart 
-4. Click checkout
-5. Enter City field empty
-6. Enter Address field empty
-7. Leave phone of reciever
-8.Enter name of reciever empty
-9. Click confirm Order button</t>
-  </si>
-  <si>
-    <t>1. Select product from home page 
-2. Add product to cart
-3. Open cart 
-4. Click checkout
-5. Enter City field empty
-6. Enter Address field empty
-7. Enter phone of reciever
-8.leave name of reciever empty
-9. Click confirm Order button</t>
-  </si>
-  <si>
-    <t>1. Select product from home page 
-2. Add product to cart
-3. Open cart 
-4. Click checkout
-5. Enter City field empty
-6. Leave Address field empty
-7. Enter phone of reciever
-8.Enter name of reciever
-9. Click confirm Order button</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Select product from home page 
-2. Add product to cart
-3. Open cart 
-4. Click checkout
-5. Leave City field empty
-6. Enter Address 
-7. Enter phone of reciever
-8.Enter name of reciever
-9. Click confirm Order button
-</t>
   </si>
   <si>
     <t>1. Select product from home page 
@@ -1507,6 +1456,59 @@
   </si>
   <si>
     <t>Verify "Back to Cart" button is displayed on the checkout page and redirects user to the cart page when clicked</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City
+6. Leave Address field empty
+7. Enter phone of reciever
+8.Enter name of reciever
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field 
+6. Enter Address field
+7. Enter phone of reciever
+8.leave name of reciever empty
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>Verify name of reciever name field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify phone of reciever phone field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field
+6. Enter Address field
+7. Leave phone of reciever
+8.Enter name of reciever 
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field 
+6. Enter Address field 
+7. Enter phone of reciever
+8.Enter name of reciever 
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify phone of reciever Phone field is mandatory when left empty with other valid data</t>
   </si>
 </sst>
 </file>
@@ -2189,7 +2191,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -2233,7 +2235,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>15</v>
@@ -2245,11 +2247,11 @@
         <v>21</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G2" s="14"/>
       <c r="H2" s="23" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="I2" s="22"/>
       <c r="J2" s="58" t="s">
@@ -2304,12 +2306,12 @@
       </c>
       <c r="N3" s="13"/>
     </row>
-    <row r="4" spans="1:27" ht="132" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
         <v>25</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
@@ -2320,8 +2322,8 @@
       <c r="E4" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="22" t="s">
-        <v>283</v>
+      <c r="F4" s="53" t="s">
+        <v>308</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="23" t="s">
@@ -2360,8 +2362,8 @@
       <c r="E5" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="22" t="s">
-        <v>282</v>
+      <c r="F5" s="53" t="s">
+        <v>316</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="23" t="s">
@@ -2389,7 +2391,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>277</v>
+        <v>318</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
@@ -2400,8 +2402,8 @@
       <c r="E6" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="22" t="s">
-        <v>281</v>
+      <c r="F6" s="53" t="s">
+        <v>317</v>
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="23" t="s">
@@ -2427,7 +2429,7 @@
         <v>28</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>279</v>
+        <v>322</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>18</v>
@@ -2438,8 +2440,8 @@
       <c r="E7" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="22" t="s">
-        <v>280</v>
+      <c r="F7" s="53" t="s">
+        <v>320</v>
       </c>
       <c r="G7" s="14"/>
       <c r="H7" s="23" t="s">
@@ -2465,7 +2467,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>15</v>
@@ -2477,11 +2479,11 @@
         <v>21</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="23" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="I8" s="22"/>
       <c r="J8" s="58" t="s">
@@ -2489,7 +2491,7 @@
       </c>
       <c r="K8" s="14"/>
       <c r="L8" s="13" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="M8" s="14" t="s">
         <v>16</v>
@@ -2500,10 +2502,10 @@
     </row>
     <row r="9" spans="1:27" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>15</v>
@@ -2515,11 +2517,11 @@
         <v>21</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="23" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="I9" s="22"/>
       <c r="J9" s="58" t="s">
@@ -2527,7 +2529,7 @@
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="13" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="M9" s="14" t="s">
         <v>16</v>
@@ -2538,7 +2540,7 @@
     </row>
     <row r="10" spans="1:27" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="B10" s="38" t="s">
         <v>29</v>
@@ -2557,11 +2559,11 @@
       </c>
       <c r="G10" s="14"/>
       <c r="H10" s="13" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="71" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="K10" s="14" t="s">
         <v>22</v>
@@ -2578,7 +2580,7 @@
     </row>
     <row r="11" spans="1:27" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="B11" s="39" t="s">
         <v>33</v>
@@ -2593,7 +2595,7 @@
         <v>21</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3" t="s">
@@ -2601,13 +2603,13 @@
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="71" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>22</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>16</v>
@@ -2631,26 +2633,26 @@
     </row>
     <row r="12" spans="1:27" ht="122.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="E12" s="41" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="58" t="s">
@@ -2660,7 +2662,7 @@
         <v>22</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>16</v>
@@ -8027,7 +8029,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="42" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="D1" s="42" t="s">
         <v>3</v>
@@ -8045,7 +8047,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="42" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="J1" s="42" t="s">
         <v>8</v>
@@ -8066,7 +8068,7 @@
         <v>13</v>
       </c>
       <c r="P1" s="43" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="Q1" s="44" t="s">
         <v>14</v>
@@ -8077,7 +8079,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C2" s="52" t="s">
         <v>15</v>
@@ -8089,16 +8091,16 @@
         <v>21</v>
       </c>
       <c r="F2" s="53" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="G2" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H2" s="51" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="I2" s="72" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="J2" s="56"/>
       <c r="K2" s="58" t="s">
@@ -8115,7 +8117,7 @@
         <v>23</v>
       </c>
       <c r="P2" s="56" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="Q2" s="56"/>
       <c r="R2" s="45"/>
@@ -8148,10 +8150,10 @@
         <v>21</v>
       </c>
       <c r="F3" s="53" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="G3" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>275</v>
@@ -8174,7 +8176,7 @@
         <v>23</v>
       </c>
       <c r="P3" s="56" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="Q3" s="56"/>
       <c r="R3" s="45"/>
@@ -8195,7 +8197,7 @@
         <v>25</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C4" s="52" t="s">
         <v>18</v>
@@ -8207,16 +8209,16 @@
         <v>26</v>
       </c>
       <c r="F4" s="53" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="G4" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H4" s="51" t="s">
         <v>270</v>
       </c>
       <c r="I4" s="51" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="J4" s="56"/>
       <c r="K4" s="58" t="s">
@@ -8233,7 +8235,7 @@
         <v>23</v>
       </c>
       <c r="P4" s="56" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="Q4" s="56"/>
       <c r="R4" s="45"/>
@@ -8266,16 +8268,16 @@
         <v>26</v>
       </c>
       <c r="F5" s="53" t="s">
-        <v>282</v>
+        <v>316</v>
       </c>
       <c r="G5" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H5" s="51" t="s">
         <v>272</v>
       </c>
       <c r="I5" s="51" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="J5" s="56"/>
       <c r="K5" s="58" t="s">
@@ -8292,7 +8294,7 @@
         <v>23</v>
       </c>
       <c r="P5" s="56" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="Q5" s="56"/>
       <c r="R5" s="45"/>
@@ -8313,7 +8315,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="57" t="s">
-        <v>277</v>
+        <v>318</v>
       </c>
       <c r="C6" s="52" t="s">
         <v>18</v>
@@ -8325,16 +8327,16 @@
         <v>21</v>
       </c>
       <c r="F6" s="53" t="s">
-        <v>281</v>
+        <v>317</v>
       </c>
       <c r="G6" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H6" s="51" t="s">
         <v>272</v>
       </c>
       <c r="I6" s="51" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="J6" s="59"/>
       <c r="K6" s="58" t="s">
@@ -8351,7 +8353,7 @@
         <v>23</v>
       </c>
       <c r="P6" s="56" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="Q6" s="61"/>
     </row>
@@ -8360,7 +8362,7 @@
         <v>28</v>
       </c>
       <c r="B7" s="57" t="s">
-        <v>279</v>
+        <v>319</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>18</v>
@@ -8372,16 +8374,16 @@
         <v>21</v>
       </c>
       <c r="F7" s="53" t="s">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="G7" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H7" s="51" t="s">
         <v>272</v>
       </c>
       <c r="I7" s="51" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="J7" s="59"/>
       <c r="K7" s="58" t="s">
@@ -8398,7 +8400,7 @@
         <v>23</v>
       </c>
       <c r="P7" s="56" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="Q7" s="61"/>
     </row>
@@ -8407,7 +8409,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="57" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>15</v>
@@ -8418,17 +8420,17 @@
       <c r="E8" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="53" t="s">
-        <v>285</v>
+      <c r="F8" s="22" t="s">
+        <v>321</v>
       </c>
       <c r="G8" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H8" s="51" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="I8" s="51" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="J8" s="59"/>
       <c r="K8" s="58" t="s">
@@ -8436,7 +8438,7 @@
       </c>
       <c r="L8" s="63"/>
       <c r="M8" s="52" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="N8" s="52" t="s">
         <v>16</v>
@@ -8445,7 +8447,7 @@
         <v>23</v>
       </c>
       <c r="P8" s="56" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="Q8" s="64"/>
       <c r="R8" s="46"/>
@@ -8463,10 +8465,10 @@
     </row>
     <row r="9" spans="1:29" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="B9" s="57" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>15</v>
@@ -8478,16 +8480,16 @@
         <v>21</v>
       </c>
       <c r="F9" s="53" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="G9" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H9" s="51" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="I9" s="51" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="J9" s="60"/>
       <c r="K9" s="58" t="s">
@@ -8495,7 +8497,7 @@
       </c>
       <c r="L9" s="60"/>
       <c r="M9" s="52" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="N9" s="52" t="s">
         <v>16</v>
@@ -8504,13 +8506,13 @@
         <v>23</v>
       </c>
       <c r="P9" s="56" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="Q9" s="61"/>
     </row>
     <row r="10" spans="1:29" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="B10" s="57" t="s">
         <v>29</v>
@@ -8528,15 +8530,15 @@
         <v>31</v>
       </c>
       <c r="G10" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H10" s="57" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="I10" s="59"/>
       <c r="J10" s="65"/>
       <c r="K10" s="71" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="L10" s="65"/>
       <c r="M10" s="67" t="s">
@@ -8565,7 +8567,7 @@
     </row>
     <row r="11" spans="1:29" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A11" s="52" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="B11" s="51" t="s">
         <v>33</v>
@@ -8580,10 +8582,10 @@
         <v>21</v>
       </c>
       <c r="F11" s="51" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="G11" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H11" s="51" t="s">
         <v>34</v>
@@ -8591,11 +8593,11 @@
       <c r="I11" s="55"/>
       <c r="J11" s="65"/>
       <c r="K11" s="71" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="L11" s="65"/>
       <c r="M11" s="52" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="N11" s="52" t="s">
         <v>16</v>
@@ -8620,31 +8622,31 @@
     </row>
     <row r="12" spans="1:29" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="52" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="B12" s="68" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="58" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="E12" s="51" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="F12" s="68" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="G12" s="54" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H12" s="68" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="I12" s="68" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="J12" s="69"/>
       <c r="K12" s="58" t="s">
@@ -8652,7 +8654,7 @@
       </c>
       <c r="L12" s="69"/>
       <c r="M12" s="52" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="N12" s="58" t="s">
         <v>16</v>
@@ -8661,7 +8663,7 @@
         <v>23</v>
       </c>
       <c r="P12" s="56" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="Q12" s="70"/>
     </row>

</xml_diff>

<commit_message>
test/update checkout execution test cases.
</commit_message>
<xml_diff>
--- a/TestCases_Docs/CHK_TCS.xlsx
+++ b/TestCases_Docs/CHK_TCS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\iti\QA\New folder\Clothing-Web-Portal\TestCases_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9236D6-EA61-4346-B3F3-1682EE664869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC662E76-20A0-4067-8400-3F73988B1D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CHK_TCS" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="323">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1732,7 +1732,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1931,6 +1931,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2602,8 +2605,8 @@
         <v>34</v>
       </c>
       <c r="I11" s="3"/>
-      <c r="J11" s="71" t="s">
-        <v>313</v>
+      <c r="J11" s="73" t="s">
+        <v>46</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>22</v>
@@ -8592,8 +8595,8 @@
       </c>
       <c r="I11" s="55"/>
       <c r="J11" s="65"/>
-      <c r="K11" s="71" t="s">
-        <v>313</v>
+      <c r="K11" s="73" t="s">
+        <v>46</v>
       </c>
       <c r="L11" s="65"/>
       <c r="M11" s="52" t="s">
@@ -8605,7 +8608,9 @@
       <c r="O11" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P11" s="56"/>
+      <c r="P11" s="56" t="s">
+        <v>306</v>
+      </c>
       <c r="Q11" s="66"/>
       <c r="R11" s="47"/>
       <c r="S11" s="47"/>

</xml_diff>

<commit_message>
test/update checkout and add test report
</commit_message>
<xml_diff>
--- a/TestCases_Docs/CHK_TCS.xlsx
+++ b/TestCases_Docs/CHK_TCS.xlsx
@@ -8,21 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\iti\QA\New folder\Clothing-Web-Portal\TestCases_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9959C0-D856-4958-B6F3-812D98494892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EDA59FB-A762-4093-8748-416C8147CDB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CHK_TCS" sheetId="2" r:id="rId1"/>
     <sheet name="CHK_TCS Execution" sheetId="4" r:id="rId2"/>
     <sheet name="Execution status v1" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="322">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1599,21 +1612,25 @@
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1626,16 +1643,19 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1729,7 +1749,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1880,9 +1900,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2251,7 +2268,7 @@
         <v>299</v>
       </c>
       <c r="I2" s="22"/>
-      <c r="J2" s="58" t="s">
+      <c r="J2" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K2" s="14" t="s">
@@ -2291,7 +2308,7 @@
         <v>275</v>
       </c>
       <c r="I3" s="22"/>
-      <c r="J3" s="58" t="s">
+      <c r="J3" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K3" s="14"/>
@@ -2327,7 +2344,7 @@
         <v>270</v>
       </c>
       <c r="I4" s="14"/>
-      <c r="J4" s="58" t="s">
+      <c r="J4" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K4" s="14" t="s">
@@ -2367,7 +2384,7 @@
         <v>272</v>
       </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="58" t="s">
+      <c r="J5" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K5" s="14" t="s">
@@ -2407,7 +2424,7 @@
         <v>272</v>
       </c>
       <c r="I6" s="14"/>
-      <c r="J6" s="58" t="s">
+      <c r="J6" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K6" s="14"/>
@@ -2445,7 +2462,7 @@
         <v>272</v>
       </c>
       <c r="I7" s="14"/>
-      <c r="J7" s="58" t="s">
+      <c r="J7" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K7" s="14"/>
@@ -2483,7 +2500,7 @@
         <v>280</v>
       </c>
       <c r="I8" s="22"/>
-      <c r="J8" s="58" t="s">
+      <c r="J8" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="14"/>
@@ -2521,7 +2538,7 @@
         <v>286</v>
       </c>
       <c r="I9" s="22"/>
-      <c r="J9" s="58" t="s">
+      <c r="J9" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K9" s="14"/>
@@ -2559,7 +2576,7 @@
         <v>289</v>
       </c>
       <c r="I10" s="14"/>
-      <c r="J10" s="71" t="s">
+      <c r="J10" s="70" t="s">
         <v>312</v>
       </c>
       <c r="K10" s="14" t="s">
@@ -2599,7 +2616,7 @@
         <v>34</v>
       </c>
       <c r="I11" s="3"/>
-      <c r="J11" s="58" t="s">
+      <c r="J11" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -2652,7 +2669,7 @@
         <v>295</v>
       </c>
       <c r="I12" s="7"/>
-      <c r="J12" s="58" t="s">
+      <c r="J12" s="57" t="s">
         <v>46</v>
       </c>
       <c r="K12" s="7" t="s">
@@ -8096,15 +8113,15 @@
       <c r="H2" s="51" t="s">
         <v>299</v>
       </c>
-      <c r="I2" s="72" t="s">
+      <c r="I2" s="71" t="s">
         <v>310</v>
       </c>
-      <c r="J2" s="56"/>
-      <c r="K2" s="58" t="s">
+      <c r="J2" s="55"/>
+      <c r="K2" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L2" s="56"/>
-      <c r="M2" s="67" t="s">
+      <c r="L2" s="55"/>
+      <c r="M2" s="66" t="s">
         <v>269</v>
       </c>
       <c r="N2" s="52" t="s">
@@ -8113,10 +8130,10 @@
       <c r="O2" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="56" t="s">
+      <c r="P2" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q2" s="56"/>
+      <c r="Q2" s="55"/>
       <c r="R2" s="45"/>
       <c r="S2" s="45"/>
       <c r="T2" s="45"/>
@@ -8158,12 +8175,12 @@
       <c r="I3" s="51" t="s">
         <v>275</v>
       </c>
-      <c r="J3" s="56"/>
-      <c r="K3" s="58" t="s">
+      <c r="J3" s="55"/>
+      <c r="K3" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L3" s="56"/>
-      <c r="M3" s="67" t="s">
+      <c r="L3" s="55"/>
+      <c r="M3" s="66" t="s">
         <v>269</v>
       </c>
       <c r="N3" s="52" t="s">
@@ -8172,10 +8189,10 @@
       <c r="O3" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P3" s="56" t="s">
+      <c r="P3" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q3" s="56"/>
+      <c r="Q3" s="55"/>
       <c r="R3" s="45"/>
       <c r="S3" s="45"/>
       <c r="T3" s="45"/>
@@ -8193,7 +8210,7 @@
       <c r="A4" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="56" t="s">
         <v>277</v>
       </c>
       <c r="C4" s="52" t="s">
@@ -8202,7 +8219,7 @@
       <c r="D4" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="57" t="s">
+      <c r="E4" s="56" t="s">
         <v>26</v>
       </c>
       <c r="F4" s="53" t="s">
@@ -8217,12 +8234,12 @@
       <c r="I4" s="51" t="s">
         <v>311</v>
       </c>
-      <c r="J4" s="56"/>
-      <c r="K4" s="58" t="s">
+      <c r="J4" s="55"/>
+      <c r="K4" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="56"/>
-      <c r="M4" s="67" t="s">
+      <c r="L4" s="55"/>
+      <c r="M4" s="66" t="s">
         <v>271</v>
       </c>
       <c r="N4" s="52" t="s">
@@ -8231,10 +8248,10 @@
       <c r="O4" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P4" s="56" t="s">
+      <c r="P4" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q4" s="56"/>
+      <c r="Q4" s="55"/>
       <c r="R4" s="45"/>
       <c r="S4" s="45"/>
       <c r="T4" s="45"/>
@@ -8252,7 +8269,7 @@
       <c r="A5" s="50" t="s">
         <v>266</v>
       </c>
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="56" t="s">
         <v>276</v>
       </c>
       <c r="C5" s="52" t="s">
@@ -8276,11 +8293,11 @@
       <c r="I5" s="51" t="s">
         <v>311</v>
       </c>
-      <c r="J5" s="56"/>
-      <c r="K5" s="58" t="s">
+      <c r="J5" s="55"/>
+      <c r="K5" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="56"/>
+      <c r="L5" s="55"/>
       <c r="M5" s="52" t="s">
         <v>268</v>
       </c>
@@ -8290,10 +8307,10 @@
       <c r="O5" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P5" s="56" t="s">
+      <c r="P5" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q5" s="56"/>
+      <c r="Q5" s="55"/>
       <c r="R5" s="45"/>
       <c r="S5" s="45"/>
       <c r="T5" s="45"/>
@@ -8311,7 +8328,7 @@
       <c r="A6" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="56" t="s">
         <v>317</v>
       </c>
       <c r="C6" s="52" t="s">
@@ -8335,11 +8352,11 @@
       <c r="I6" s="51" t="s">
         <v>311</v>
       </c>
-      <c r="J6" s="59"/>
-      <c r="K6" s="58" t="s">
+      <c r="J6" s="58"/>
+      <c r="K6" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L6" s="60"/>
+      <c r="L6" s="59"/>
       <c r="M6" s="52" t="s">
         <v>268</v>
       </c>
@@ -8349,16 +8366,16 @@
       <c r="O6" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P6" s="56" t="s">
+      <c r="P6" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q6" s="61"/>
+      <c r="Q6" s="60"/>
     </row>
     <row r="7" spans="1:29" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="56" t="s">
         <v>318</v>
       </c>
       <c r="C7" s="52" t="s">
@@ -8382,11 +8399,11 @@
       <c r="I7" s="51" t="s">
         <v>311</v>
       </c>
-      <c r="J7" s="59"/>
-      <c r="K7" s="58" t="s">
+      <c r="J7" s="58"/>
+      <c r="K7" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L7" s="60"/>
+      <c r="L7" s="59"/>
       <c r="M7" s="52" t="s">
         <v>268</v>
       </c>
@@ -8396,16 +8413,16 @@
       <c r="O7" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P7" s="56" t="s">
+      <c r="P7" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q7" s="61"/>
+      <c r="Q7" s="60"/>
     </row>
     <row r="8" spans="1:29" ht="118.8" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="56" t="s">
         <v>282</v>
       </c>
       <c r="C8" s="52" t="s">
@@ -8414,7 +8431,7 @@
       <c r="D8" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="62" t="s">
+      <c r="E8" s="61" t="s">
         <v>21</v>
       </c>
       <c r="F8" s="22" t="s">
@@ -8429,11 +8446,11 @@
       <c r="I8" s="51" t="s">
         <v>280</v>
       </c>
-      <c r="J8" s="59"/>
-      <c r="K8" s="58" t="s">
+      <c r="J8" s="58"/>
+      <c r="K8" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L8" s="63"/>
+      <c r="L8" s="62"/>
       <c r="M8" s="52" t="s">
         <v>281</v>
       </c>
@@ -8443,10 +8460,10 @@
       <c r="O8" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P8" s="56" t="s">
+      <c r="P8" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q8" s="64"/>
+      <c r="Q8" s="63"/>
       <c r="R8" s="46"/>
       <c r="S8" s="46"/>
       <c r="T8" s="46"/>
@@ -8464,7 +8481,7 @@
       <c r="A9" s="50" t="s">
         <v>283</v>
       </c>
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="56" t="s">
         <v>313</v>
       </c>
       <c r="C9" s="52" t="s">
@@ -8473,7 +8490,7 @@
       <c r="D9" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="62" t="s">
+      <c r="E9" s="61" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="53" t="s">
@@ -8488,11 +8505,11 @@
       <c r="I9" s="51" t="s">
         <v>286</v>
       </c>
-      <c r="J9" s="60"/>
-      <c r="K9" s="58" t="s">
+      <c r="J9" s="59"/>
+      <c r="K9" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="60"/>
+      <c r="L9" s="59"/>
       <c r="M9" s="52" t="s">
         <v>287</v>
       </c>
@@ -8502,16 +8519,16 @@
       <c r="O9" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P9" s="56" t="s">
+      <c r="P9" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q9" s="61"/>
+      <c r="Q9" s="60"/>
     </row>
     <row r="10" spans="1:29" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
         <v>288</v>
       </c>
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="56" t="s">
         <v>29</v>
       </c>
       <c r="C10" s="52" t="s">
@@ -8520,7 +8537,7 @@
       <c r="D10" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="57" t="s">
+      <c r="E10" s="56" t="s">
         <v>30</v>
       </c>
       <c r="F10" s="53" t="s">
@@ -8529,16 +8546,16 @@
       <c r="G10" s="54" t="s">
         <v>304</v>
       </c>
-      <c r="H10" s="57" t="s">
+      <c r="H10" s="56" t="s">
         <v>289</v>
       </c>
-      <c r="I10" s="59"/>
-      <c r="J10" s="65"/>
-      <c r="K10" s="71" t="s">
+      <c r="I10" s="58"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="70" t="s">
         <v>312</v>
       </c>
-      <c r="L10" s="65"/>
-      <c r="M10" s="67" t="s">
+      <c r="L10" s="64"/>
+      <c r="M10" s="66" t="s">
         <v>267</v>
       </c>
       <c r="N10" s="52" t="s">
@@ -8547,8 +8564,10 @@
       <c r="O10" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="66"/>
+      <c r="P10" s="70" t="s">
+        <v>312</v>
+      </c>
+      <c r="Q10" s="65"/>
       <c r="R10" s="47"/>
       <c r="S10" s="47"/>
       <c r="T10" s="47"/>
@@ -8587,12 +8606,14 @@
       <c r="H11" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="I11" s="55"/>
-      <c r="J11" s="65"/>
-      <c r="K11" s="58" t="s">
+      <c r="I11" s="51" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="64"/>
+      <c r="K11" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="65"/>
+      <c r="L11" s="64"/>
       <c r="M11" s="52" t="s">
         <v>291</v>
       </c>
@@ -8602,10 +8623,10 @@
       <c r="O11" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="P11" s="56" t="s">
+      <c r="P11" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q11" s="66"/>
+      <c r="Q11" s="65"/>
       <c r="R11" s="47"/>
       <c r="S11" s="47"/>
       <c r="T11" s="47"/>
@@ -8623,48 +8644,48 @@
       <c r="A12" s="52" t="s">
         <v>296</v>
       </c>
-      <c r="B12" s="68" t="s">
+      <c r="B12" s="67" t="s">
         <v>314</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="58" t="s">
+      <c r="D12" s="57" t="s">
         <v>293</v>
       </c>
       <c r="E12" s="51" t="s">
         <v>294</v>
       </c>
-      <c r="F12" s="68" t="s">
+      <c r="F12" s="67" t="s">
         <v>308</v>
       </c>
       <c r="G12" s="54" t="s">
         <v>304</v>
       </c>
-      <c r="H12" s="68" t="s">
+      <c r="H12" s="67" t="s">
         <v>295</v>
       </c>
-      <c r="I12" s="68" t="s">
+      <c r="I12" s="67" t="s">
         <v>295</v>
       </c>
-      <c r="J12" s="69"/>
-      <c r="K12" s="58" t="s">
+      <c r="J12" s="68"/>
+      <c r="K12" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="L12" s="69"/>
+      <c r="L12" s="68"/>
       <c r="M12" s="52" t="s">
         <v>298</v>
       </c>
-      <c r="N12" s="58" t="s">
+      <c r="N12" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="O12" s="58" t="s">
+      <c r="O12" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="P12" s="56" t="s">
+      <c r="P12" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="Q12" s="70"/>
+      <c r="Q12" s="69"/>
     </row>
     <row r="13" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F13" s="48"/>
@@ -14135,7 +14156,7 @@
       <c r="Q988" s="48"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="P2:P12">
+  <conditionalFormatting sqref="P2:P9 P11:P12">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",P2)))</formula>
     </cfRule>
@@ -14147,10 +14168,10 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C12" xr:uid="{3CFE6C65-50FD-4F47-8059-264292110C82}">
       <formula1>"valid,invalid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P12" xr:uid="{9A74E543-1C36-40E5-9DBB-0F7FF27E4F62}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P9 P11:P12" xr:uid="{9A74E543-1C36-40E5-9DBB-0F7FF27E4F62}">
       <formula1>"Passed, Failed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2:K12" xr:uid="{C4EE6916-F62E-4448-8961-4E20989DF001}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2:K12 P10" xr:uid="{C4EE6916-F62E-4448-8961-4E20989DF001}">
       <formula1>"in progress,in review,approved,cancelled"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>